<commit_message>
docs(authoring): apply teacher's paper-book rulings on 3 ambiguous page-map rows (final 127✓/25✗/0؟)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/authoring/PAGE-MAP-KH-G2-MATH-v1_verified.xlsx
+++ b/authoring/PAGE-MAP-KH-G2-MATH-v1_verified.xlsx
@@ -1293,17 +1293,17 @@
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>؟</t>
+          <t>✗</t>
         </is>
       </c>
       <c r="O11" s="7" t="inlineStr">
         <is>
-          <t>(الف) ادعای «۸ شکل» با جدول شمارش ۵ستونه (۵ نوع گل) نمی‌خواند — تصویر جدول ۵ ستون دارد. (ب) «جدول شگفت‌انگیز» فیل خانه‌هایی با عددهای دو رقمی (۲۵، ۵۹، ۸۵ و…) دارد و توصیف «عددهای ۱ تا ۹» قطعی نیست. نیازمند حکم کتاب کاغذی.</t>
+          <t>ساختار طبق حکم کتاب کاغذی تأیید شد: فعّالیت دو نفرهٔ شمارش چوب‌خط (بالای صفحه) + «جدول شگفت‌انگیز» (زیر آن). دو مقدار اصلاح می‌شود: (۱) جدول شمارش ۵ ستون دارد (۵ نوع گل: نیلوفر، گل لیوانی، لاله، غنچه، گل سفید) — نه «۸ شکل». (۲) جدول شگفت‌انگیز فیل شبکهٔ ۸×۸ از عددهای یک‌رقمی و دو رقمی (تا ۸۵) با خانه‌های خالی است — توصیف «عددهای ۱ تا ۹» دقیق نیست.</t>
         </is>
       </c>
       <c r="P11" s="5" t="inlineStr">
         <is>
-          <t>PDF ۹ (ص کتاب ۳): جدول گل‌ها (وسط صفحه) + جدول شگفت‌انگیز فیل (پایین) — تأیید با عکس کتاب کاغذی</t>
+          <t>PDF ۹ (ص کتاب ۳): جدول شمارش (وسط صفحه) + جدول شگفت‌انگیز فیل (پایین) — تأیید با کتاب کاغذی معلّم</t>
         </is>
       </c>
     </row>
@@ -10405,17 +10405,17 @@
       </c>
       <c r="N137" s="5" t="inlineStr">
         <is>
-          <t>؟</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="O137" s="7" t="inlineStr">
         <is>
-          <t>مقادیر جدول «رضا» (ساعت‌های انجام تکالیف هر روز) و «جمع ۱۸ ساعت» از روی تصویر قطعی نیست؛ خوانش من از جدول مقادیری نزدیک به ۲ (و یک ۱) نشان می‌دهد که با جمع ۱۸ نمی‌خواند. جدول «سارا» (چوب‌خط‌های کار خوب هر روز) نیز به شمارش تصویری دقیق نیاز دارد. نیازمند حکم کتاب کاغذی. ساختار صفحه ✓ (دو مورد شماره‌دار + سه پرسش).</t>
+          <t>—</t>
         </is>
       </c>
       <c r="P137" s="5" t="inlineStr">
         <is>
-          <t>PDF ۱۳۵ (ص کتاب ۱۲۹): دو جدول وسط/پایین صفحه</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -10976,17 +10976,17 @@
       </c>
       <c r="N145" s="5" t="inlineStr">
         <is>
-          <t>؟</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="O145" s="7" t="inlineStr">
         <is>
-          <t>مقادیر چاپی جدول خیابان‌ها و شمارش فلش‌های «نمودار توری» با خوانش تصویری من قطعی نشد: نقشه برای انقلاب/آزادی «۴۰/۶۰» می‌گوید و خوانش من از تصویر با آن نمی‌خواند؛ برای ردیف‌های استقلال/امام رضا تصویر ~۶ فلش و ~۵ فلش (هر فلش = ۱۰ خانه) نشان می‌دهد ولی عدد چاپی ندارند. ساختار صفحه ✓ (دو مورد شماره‌دار + جدول + نمودار). نیازمند حکم کتاب کاغذی.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="P145" s="5" t="inlineStr">
         <is>
-          <t>PDF ۱۴۳ (ص کتاب ۱۳۷): جدول خیابان‌ها + ستون نمودار توری</t>
+          <t>—</t>
         </is>
       </c>
     </row>

</xml_diff>